<commit_message>
Fix mailing and homepage
</commit_message>
<xml_diff>
--- a/event_list.xlsx
+++ b/event_list.xlsx
@@ -122,12 +122,12 @@
       <alignment vertical="top"/>
       <protection hidden="0" locked="1"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top"/>
+      <protection hidden="0" locked="1"/>
+    </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
-      <protection hidden="0" locked="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top"/>
       <protection hidden="0" locked="1"/>
     </xf>
   </cellXfs>
@@ -632,8 +632,8 @@
       </c>
     </row>
     <row r="2" ht="102">
-      <c r="A2" s="2">
-        <v>46377</v>
+      <c r="A2" s="4">
+        <v>46306</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>6</v>
@@ -647,13 +647,16 @@
       <c r="E2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="5" t="s">
         <v>10</v>
       </c>
+      <c r="G2"/>
+      <c r="H2"/>
+      <c r="I2"/>
     </row>
     <row r="3" ht="102">
-      <c r="A3" s="5">
-        <v>46290</v>
+      <c r="A3" s="2">
+        <v>46054</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>6</v>
@@ -667,35 +670,15 @@
       <c r="E3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="5" t="s">
         <v>10</v>
       </c>
       <c r="G3"/>
       <c r="H3"/>
       <c r="I3"/>
     </row>
-    <row r="4" ht="102">
-      <c r="A4" s="2">
-        <v>46185</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G4"/>
-      <c r="H4"/>
-      <c r="I4"/>
+    <row r="4" ht="12.75">
+      <c r="A4" s="1"/>
     </row>
     <row r="5" ht="12.75">
       <c r="A5" s="1"/>
@@ -723,9 +706,6 @@
     </row>
     <row r="13" ht="12.75">
       <c r="A13" s="1"/>
-    </row>
-    <row r="14" ht="12.75">
-      <c r="A14" s="1"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>

</xml_diff>

<commit_message>
Add events in the list
</commit_message>
<xml_diff>
--- a/event_list.xlsx
+++ b/event_list.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>date</t>
   </si>
@@ -37,23 +37,43 @@
     <t>details</t>
   </si>
   <si>
-    <t>Colloquium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">What even is redundancy and deficiency?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Name, Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">University of Vienna · University of Graz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">**Time:** 09:00-17:00  
-**Location:** Seminar Room 14, University of Vienna
-This workshop examines the interaction between redundancy and deficiency across different linguistic domains.
-[View programme](events/programmes/workshop-name.pdf){.event-link}
-</t>
+    <t>Workshop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clitic Meeting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anita Riedl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">University of Salzburg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">**Date:** October 29-30&lt;br&gt;
+**Location:** University of Salzburg&lt;br&gt;
+&lt;br&gt;
+This workshop examines clitics.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Current Issues in Syntax, Semantics, and Pragmatics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">**Date:** November 20-21&lt;br&gt;
+**Location:** University of Salzburg&lt;br&gt;
+&lt;br&gt;
+Fourth edition of the 'Current Issues in Syntax, Semantics, and Pragmatics' workshop&lt;br&gt;
+&lt;br&gt;
+Contact email: synsemprag.workshop@gmail.com&lt;br&gt;
+[Page of the conference](https://www.plus.ac.at/linguistik/tagungen-und-vortraege/tagungen/){.event-link}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SFB Retreat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">**Date:** June 17-19&lt;br&gt;
+**Location:** Sport Hotel Kapfenberg&lt;br&gt;
+&lt;br&gt;
+Third edition of the SFB retreat.&lt;br&gt;</t>
   </si>
 </sst>
 </file>
@@ -107,7 +127,7 @@
     <xf fontId="1" fillId="0" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
     <xf fontId="2" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyProtection="0">
       <protection hidden="0" locked="1"/>
     </xf>
@@ -123,6 +143,10 @@
       <protection hidden="0" locked="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top"/>
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="top"/>
       <protection hidden="0" locked="1"/>
     </xf>
@@ -631,54 +655,54 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" ht="102">
+    <row r="2" ht="63.75">
       <c r="A2" s="4">
-        <v>46306</v>
-      </c>
-      <c r="B2" s="3" t="s">
+        <v>46324</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="G2"/>
-      <c r="H2"/>
-      <c r="I2"/>
     </row>
     <row r="3" ht="102">
       <c r="A3" s="2">
-        <v>46054</v>
-      </c>
-      <c r="B3" s="3" t="s">
+        <v>46346</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>8</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="D3" s="3"/>
       <c r="E3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="G3"/>
-      <c r="H3"/>
-      <c r="I3"/>
-    </row>
-    <row r="4" ht="12.75">
-      <c r="A4" s="1"/>
+      <c r="F3" s="6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" ht="51">
+      <c r="A4" s="1">
+        <v>46190</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="5" ht="12.75">
       <c r="A5" s="1"/>

</xml_diff>

<commit_message>
Fix bibtex keys and event links
</commit_message>
<xml_diff>
--- a/event_list.xlsx
+++ b/event_list.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>date</t>
   </si>
@@ -58,7 +58,7 @@
 **Location:** University of Salzburg
 Fourth edition of the 'Current Issues in Syntax, Semantics, and Pragmatics' workshop
 Contact email: synsemprag.workshop@gmail.com
-[Page of the conference](https://www.plus.ac.at/linguistik/tagungen-und-vortraege/tagungen/){.event-link}</t>
+[Page of the conference](https://www.plus.ac.at/linguistik/tagungen-und-vortraege/tagungen/)</t>
   </si>
   <si>
     <t xml:space="preserve">SFB Retreat</t>
@@ -70,20 +70,6 @@
     <t xml:space="preserve">**Date:** June 17-19
 **Location:** Sport Hotel Kapfenberg
 Third edition of the SFB retreat.</t>
-  </si>
-  <si>
-    <t>Talk</t>
-  </si>
-  <si>
-    <t xml:space="preserve">What is redundancy?</t>
-  </si>
-  <si>
-    <t>Edgar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">**Date:** October 30, 11:00-13:00
-Click [here](https://github.io/yanhiz/sfb_redefi){.event-link}
-</t>
   </si>
 </sst>
 </file>
@@ -149,7 +135,7 @@
     <xf fontId="1" fillId="0" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
     <xf fontId="2" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyProtection="0">
       <protection hidden="0" locked="1"/>
     </xf>
@@ -192,13 +178,6 @@
     </xf>
     <xf fontId="0" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
-      <protection hidden="0" locked="1"/>
-    </xf>
-    <xf fontId="0" fillId="2" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1" applyFill="1" applyProtection="0">
-      <protection hidden="0" locked="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1" applyProtection="0">
-      <alignment wrapText="1"/>
       <protection hidden="0" locked="1"/>
     </xf>
   </cellXfs>
@@ -752,29 +731,14 @@
       <c r="E4" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="11" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" ht="51">
-      <c r="A5" s="12">
-        <v>46325</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F5" s="13" t="s">
-        <v>18</v>
-      </c>
+    <row r="5" ht="12.75">
+      <c r="A5" s="1"/>
+      <c r="C5"/>
+      <c r="F5"/>
     </row>
     <row r="6" ht="12.75">
       <c r="A6" s="1"/>
@@ -796,9 +760,6 @@
     </row>
     <row r="12" ht="12.75">
       <c r="A12" s="1"/>
-    </row>
-    <row r="13" ht="12.75">
-      <c r="A13" s="1"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>

</xml_diff>